<commit_message>
I thikn i worked on a bunch of GHG stuff
</commit_message>
<xml_diff>
--- a/Data/Flux_Calc/GC_Data/Belt_Data/batch_47_21_belt_data.xlsx
+++ b/Data/Flux_Calc/GC_Data/Belt_Data/batch_47_21_belt_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/telharehman/Desktop/Staff Research Associate/Projects/AWD-GHG/Analysis/AWD-GHG/DATA/0_batch2input/belt_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhang\Documents\GitHub\Sulfate_Drain\Data\Flux_Calc\GC_Data\Belt_Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC5A0BD1-856B-1444-A526-1C3DFBBFAF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DB08BCB-7347-4894-B872-4E9849B39E47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="251" uniqueCount="23">
   <si>
     <t>sample_type</t>
   </si>
@@ -377,14 +377,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K1000"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:K989"/>
+  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="11" width="25.1640625" customWidth="1"/>
+    <col min="1" max="11" width="25.125" customWidth="1"/>
     <col min="12" max="26" width="10.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -419,7 +419,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
@@ -442,7 +442,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -465,7 +465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
@@ -488,7 +488,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>11</v>
       </c>
@@ -511,7 +511,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
@@ -534,7 +534,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -557,7 +557,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
@@ -580,7 +580,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -603,7 +603,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
@@ -626,7 +626,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>20</v>
       </c>
@@ -657,7 +657,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
@@ -688,7 +688,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>20</v>
       </c>
@@ -719,7 +719,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>20</v>
       </c>
@@ -750,7 +750,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>20</v>
       </c>
@@ -781,7 +781,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>20</v>
       </c>
@@ -812,7 +812,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>20</v>
       </c>
@@ -843,7 +843,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>20</v>
       </c>
@@ -874,7 +874,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -897,7 +897,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>20</v>
       </c>
@@ -928,7 +928,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
@@ -959,7 +959,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -990,7 +990,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>20</v>
       </c>
@@ -1021,7 +1021,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>20</v>
       </c>
@@ -1052,7 +1052,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>20</v>
       </c>
@@ -1083,7 +1083,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>20</v>
       </c>
@@ -1114,7 +1114,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>20</v>
       </c>
@@ -1145,7 +1145,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -1168,7 +1168,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>20</v>
       </c>
@@ -1199,7 +1199,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>20</v>
       </c>
@@ -1230,7 +1230,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>20</v>
       </c>
@@ -1261,7 +1261,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>20</v>
       </c>
@@ -1292,7 +1292,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>20</v>
       </c>
@@ -1323,7 +1323,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>20</v>
       </c>
@@ -1354,7 +1354,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>20</v>
       </c>
@@ -1385,7 +1385,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>20</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>11</v>
       </c>
@@ -1439,7 +1439,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>20</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>20</v>
       </c>
@@ -1501,7 +1501,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>20</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>20</v>
       </c>
@@ -1563,7 +1563,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>20</v>
       </c>
@@ -1594,7 +1594,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>20</v>
       </c>
@@ -1625,7 +1625,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>20</v>
       </c>
@@ -1656,7 +1656,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>20</v>
       </c>
@@ -1687,7 +1687,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>11</v>
       </c>
@@ -1710,7 +1710,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>20</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>20</v>
       </c>
@@ -1772,7 +1772,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>20</v>
       </c>
@@ -1803,7 +1803,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>20</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>20</v>
       </c>
@@ -1865,7 +1865,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>20</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>20</v>
       </c>
@@ -1927,7 +1927,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="54" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>20</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="55" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>11</v>
       </c>
@@ -1981,7 +1981,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>20</v>
       </c>
@@ -2012,7 +2012,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>20</v>
       </c>
@@ -2043,7 +2043,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>20</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>20</v>
       </c>
@@ -2105,7 +2105,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>20</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>20</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>20</v>
       </c>
@@ -2198,7 +2198,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>20</v>
       </c>
@@ -2229,7 +2229,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>11</v>
       </c>
@@ -2252,7 +2252,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>20</v>
       </c>
@@ -2283,7 +2283,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>20</v>
       </c>
@@ -2314,7 +2314,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>20</v>
       </c>
@@ -2345,7 +2345,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>20</v>
       </c>
@@ -2376,7 +2376,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>20</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>20</v>
       </c>
@@ -2438,7 +2438,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>20</v>
       </c>
@@ -2469,7 +2469,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>20</v>
       </c>
@@ -2500,7 +2500,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>11</v>
       </c>
@@ -2523,7 +2523,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="74" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>20</v>
       </c>
@@ -2554,7 +2554,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>20</v>
       </c>
@@ -2585,7 +2585,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>20</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>20</v>
       </c>
@@ -2647,7 +2647,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>20</v>
       </c>
@@ -2678,7 +2678,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>20</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="80" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>20</v>
       </c>
@@ -2740,7 +2740,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="81" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>20</v>
       </c>
@@ -2771,1776 +2771,1459 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B82" s="1">
-        <v>93</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="E82" s="2"/>
-      <c r="F82" s="2"/>
-      <c r="G82" s="2"/>
-      <c r="H82" s="1"/>
-      <c r="I82" s="1"/>
-      <c r="J82" s="1"/>
-      <c r="K82" s="1">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B83" s="1">
-        <v>94</v>
-      </c>
-      <c r="C83" s="1"/>
-      <c r="D83" s="1"/>
-      <c r="E83" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F83" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G83" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H83" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I83" s="1">
-        <v>305</v>
-      </c>
-      <c r="J83" s="1">
-        <v>0</v>
-      </c>
-      <c r="K83" s="1">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B84" s="1">
-        <v>95</v>
-      </c>
-      <c r="C84" s="1"/>
-      <c r="D84" s="1"/>
-      <c r="E84" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F84" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G84" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H84" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I84" s="1">
-        <v>305</v>
-      </c>
-      <c r="J84" s="1">
-        <v>21</v>
-      </c>
-      <c r="K84" s="1">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B85" s="1">
-        <v>96</v>
-      </c>
-      <c r="C85" s="1"/>
-      <c r="D85" s="1"/>
-      <c r="E85" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F85" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G85" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H85" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I85" s="1">
-        <v>305</v>
-      </c>
-      <c r="J85" s="1">
-        <v>42</v>
-      </c>
-      <c r="K85" s="1">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B86" s="1">
-        <v>97</v>
-      </c>
-      <c r="C86" s="1"/>
-      <c r="D86" s="1"/>
-      <c r="E86" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F86" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G86" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H86" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I86" s="1">
-        <v>305</v>
-      </c>
-      <c r="J86" s="1">
-        <v>63</v>
-      </c>
-      <c r="K86" s="1">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B87" s="1">
-        <v>98</v>
-      </c>
-      <c r="C87" s="1"/>
-      <c r="D87" s="1"/>
-      <c r="E87" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F87" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G87" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H87" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I87" s="1">
-        <v>306</v>
-      </c>
-      <c r="J87" s="1">
-        <v>0</v>
-      </c>
-      <c r="K87" s="1">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B88" s="1">
-        <v>99</v>
-      </c>
-      <c r="C88" s="1"/>
-      <c r="D88" s="1"/>
-      <c r="E88" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F88" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G88" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H88" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I88" s="1">
-        <v>306</v>
-      </c>
-      <c r="J88" s="1">
-        <v>21</v>
-      </c>
-      <c r="K88" s="1">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="89" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B89" s="1">
-        <v>100</v>
-      </c>
-      <c r="C89" s="1"/>
-      <c r="D89" s="1"/>
-      <c r="E89" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F89" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G89" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H89" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I89" s="1">
-        <v>306</v>
-      </c>
-      <c r="J89" s="1">
-        <v>42</v>
-      </c>
-      <c r="K89" s="1">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="90" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B90" s="1">
-        <v>101</v>
-      </c>
-      <c r="C90" s="1"/>
-      <c r="D90" s="1"/>
-      <c r="E90" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F90" s="2">
-        <v>45818</v>
-      </c>
-      <c r="G90" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H90" s="1">
-        <v>2025</v>
-      </c>
-      <c r="I90" s="1">
-        <v>306</v>
-      </c>
-      <c r="J90" s="1">
-        <v>63</v>
-      </c>
-      <c r="K90" s="1">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="91" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B91" s="1">
-        <v>102</v>
-      </c>
-      <c r="C91" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="E91" s="1"/>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-      <c r="H91" s="1"/>
-      <c r="I91" s="1"/>
-      <c r="J91" s="1"/>
-      <c r="K91" s="1">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="92" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B92" s="1">
-        <v>103</v>
-      </c>
-      <c r="C92" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E92" s="1"/>
-      <c r="F92" s="2"/>
-      <c r="G92" s="2"/>
-      <c r="H92" s="1"/>
-      <c r="I92" s="1"/>
-      <c r="J92" s="1"/>
-      <c r="K92" s="1">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="93" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="94" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="97" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="98" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="99" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="100" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="101" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="102" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="103" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="104" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="105" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="106" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="107" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="108" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="109" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="110" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="111" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="112" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="113" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="114" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="115" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="116" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="117" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="83" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="84" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="85" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="87" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="88" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="89" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="90" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="91" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="92" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="93" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="94" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="95" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="96" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="97" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="98" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="99" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="100" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="101" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="102" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="103" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="104" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="105" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="106" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F106" s="3"/>
+      <c r="G106" s="3"/>
+    </row>
+    <row r="107" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F107" s="3"/>
+      <c r="G107" s="3"/>
+    </row>
+    <row r="108" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F108" s="3"/>
+      <c r="G108" s="3"/>
+    </row>
+    <row r="109" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F109" s="3"/>
+      <c r="G109" s="3"/>
+    </row>
+    <row r="110" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F110" s="3"/>
+      <c r="G110" s="3"/>
+    </row>
+    <row r="111" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F111" s="3"/>
+      <c r="G111" s="3"/>
+    </row>
+    <row r="112" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F112" s="3"/>
+      <c r="G112" s="3"/>
+    </row>
+    <row r="113" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F113" s="3"/>
+      <c r="G113" s="3"/>
+    </row>
+    <row r="114" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F114" s="3"/>
+      <c r="G114" s="3"/>
+    </row>
+    <row r="115" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F115" s="3"/>
+      <c r="G115" s="3"/>
+    </row>
+    <row r="116" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E116" s="3"/>
+      <c r="F116" s="3"/>
+      <c r="G116" s="3"/>
+    </row>
+    <row r="117" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F117" s="3"/>
       <c r="G117" s="3"/>
     </row>
-    <row r="118" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F118" s="3"/>
       <c r="G118" s="3"/>
     </row>
-    <row r="119" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F119" s="3"/>
       <c r="G119" s="3"/>
     </row>
-    <row r="120" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F120" s="3"/>
       <c r="G120" s="3"/>
     </row>
-    <row r="121" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F121" s="3"/>
       <c r="G121" s="3"/>
     </row>
-    <row r="122" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F122" s="3"/>
       <c r="G122" s="3"/>
     </row>
-    <row r="123" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F123" s="3"/>
       <c r="G123" s="3"/>
     </row>
-    <row r="124" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F124" s="3"/>
       <c r="G124" s="3"/>
     </row>
-    <row r="125" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F125" s="3"/>
       <c r="G125" s="3"/>
     </row>
-    <row r="126" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F126" s="3"/>
       <c r="G126" s="3"/>
     </row>
-    <row r="127" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E127" s="3"/>
+    <row r="127" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F127" s="3"/>
       <c r="G127" s="3"/>
     </row>
-    <row r="128" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F128" s="3"/>
       <c r="G128" s="3"/>
     </row>
-    <row r="129" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F129" s="3"/>
       <c r="G129" s="3"/>
     </row>
-    <row r="130" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F130" s="3"/>
       <c r="G130" s="3"/>
     </row>
-    <row r="131" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F131" s="3"/>
       <c r="G131" s="3"/>
     </row>
-    <row r="132" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F132" s="3"/>
       <c r="G132" s="3"/>
     </row>
-    <row r="133" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F133" s="3"/>
       <c r="G133" s="3"/>
     </row>
-    <row r="134" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E134" s="3"/>
       <c r="F134" s="3"/>
       <c r="G134" s="3"/>
     </row>
-    <row r="135" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F135" s="3"/>
       <c r="G135" s="3"/>
     </row>
-    <row r="136" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F136" s="3"/>
       <c r="G136" s="3"/>
     </row>
-    <row r="137" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F137" s="3"/>
       <c r="G137" s="3"/>
     </row>
-    <row r="138" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F138" s="3"/>
       <c r="G138" s="3"/>
     </row>
-    <row r="139" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F139" s="3"/>
       <c r="G139" s="3"/>
     </row>
-    <row r="140" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F140" s="3"/>
       <c r="G140" s="3"/>
     </row>
-    <row r="141" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F141" s="3"/>
       <c r="G141" s="3"/>
     </row>
-    <row r="142" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F142" s="3"/>
       <c r="G142" s="3"/>
     </row>
-    <row r="143" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F143" s="3"/>
       <c r="G143" s="3"/>
     </row>
-    <row r="144" spans="6:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F144" s="3"/>
       <c r="G144" s="3"/>
     </row>
-    <row r="145" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E145" s="3"/>
+    <row r="145" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F145" s="3"/>
       <c r="G145" s="3"/>
     </row>
-    <row r="146" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F146" s="3"/>
       <c r="G146" s="3"/>
     </row>
-    <row r="147" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F147" s="3"/>
       <c r="G147" s="3"/>
     </row>
-    <row r="148" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F148" s="3"/>
       <c r="G148" s="3"/>
     </row>
-    <row r="149" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F149" s="3"/>
       <c r="G149" s="3"/>
     </row>
-    <row r="150" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F150" s="3"/>
       <c r="G150" s="3"/>
     </row>
-    <row r="151" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F151" s="3"/>
       <c r="G151" s="3"/>
     </row>
-    <row r="152" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E152" s="3"/>
       <c r="F152" s="3"/>
       <c r="G152" s="3"/>
     </row>
-    <row r="153" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F153" s="3"/>
       <c r="G153" s="3"/>
     </row>
-    <row r="154" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F154" s="3"/>
       <c r="G154" s="3"/>
     </row>
-    <row r="155" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F155" s="3"/>
       <c r="G155" s="3"/>
     </row>
-    <row r="156" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F156" s="3"/>
       <c r="G156" s="3"/>
     </row>
-    <row r="157" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F157" s="3"/>
       <c r="G157" s="3"/>
     </row>
-    <row r="158" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F158" s="3"/>
       <c r="G158" s="3"/>
     </row>
-    <row r="159" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F159" s="3"/>
       <c r="G159" s="3"/>
     </row>
-    <row r="160" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F160" s="3"/>
       <c r="G160" s="3"/>
     </row>
-    <row r="161" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E161" s="3"/>
       <c r="F161" s="3"/>
       <c r="G161" s="3"/>
     </row>
-    <row r="162" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F162" s="3"/>
       <c r="G162" s="3"/>
     </row>
-    <row r="163" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E163" s="3"/>
+    <row r="163" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F163" s="3"/>
       <c r="G163" s="3"/>
     </row>
-    <row r="164" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F164" s="3"/>
       <c r="G164" s="3"/>
     </row>
-    <row r="165" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F165" s="3"/>
       <c r="G165" s="3"/>
     </row>
-    <row r="166" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F166" s="3"/>
       <c r="G166" s="3"/>
     </row>
-    <row r="167" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F167" s="3"/>
       <c r="G167" s="3"/>
     </row>
-    <row r="168" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F168" s="3"/>
       <c r="G168" s="3"/>
     </row>
-    <row r="169" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F169" s="3"/>
       <c r="G169" s="3"/>
     </row>
-    <row r="170" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E170" s="3"/>
       <c r="F170" s="3"/>
       <c r="G170" s="3"/>
     </row>
-    <row r="171" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F171" s="3"/>
       <c r="G171" s="3"/>
     </row>
-    <row r="172" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E172" s="3"/>
+    <row r="172" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F172" s="3"/>
       <c r="G172" s="3"/>
     </row>
-    <row r="173" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F173" s="3"/>
       <c r="G173" s="3"/>
     </row>
-    <row r="174" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F174" s="3"/>
       <c r="G174" s="3"/>
     </row>
-    <row r="175" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F175" s="3"/>
       <c r="G175" s="3"/>
     </row>
-    <row r="176" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F176" s="3"/>
       <c r="G176" s="3"/>
     </row>
-    <row r="177" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F177" s="3"/>
       <c r="G177" s="3"/>
     </row>
-    <row r="178" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F178" s="3"/>
       <c r="G178" s="3"/>
     </row>
-    <row r="179" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E179" s="3"/>
       <c r="F179" s="3"/>
       <c r="G179" s="3"/>
     </row>
-    <row r="180" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F180" s="3"/>
       <c r="G180" s="3"/>
     </row>
-    <row r="181" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E181" s="3"/>
+    <row r="181" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F181" s="3"/>
       <c r="G181" s="3"/>
     </row>
-    <row r="182" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F182" s="3"/>
       <c r="G182" s="3"/>
     </row>
-    <row r="183" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F183" s="3"/>
       <c r="G183" s="3"/>
     </row>
-    <row r="184" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F184" s="3"/>
       <c r="G184" s="3"/>
     </row>
-    <row r="185" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F185" s="3"/>
       <c r="G185" s="3"/>
     </row>
-    <row r="186" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F186" s="3"/>
       <c r="G186" s="3"/>
     </row>
-    <row r="187" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F187" s="3"/>
       <c r="G187" s="3"/>
     </row>
-    <row r="188" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E188" s="3"/>
       <c r="F188" s="3"/>
       <c r="G188" s="3"/>
     </row>
-    <row r="189" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F189" s="3"/>
       <c r="G189" s="3"/>
     </row>
-    <row r="190" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E190" s="3"/>
+    <row r="190" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F190" s="3"/>
       <c r="G190" s="3"/>
     </row>
-    <row r="191" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F191" s="3"/>
       <c r="G191" s="3"/>
     </row>
-    <row r="192" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F192" s="3"/>
       <c r="G192" s="3"/>
     </row>
-    <row r="193" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F193" s="3"/>
       <c r="G193" s="3"/>
     </row>
-    <row r="194" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F194" s="3"/>
       <c r="G194" s="3"/>
     </row>
-    <row r="195" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F195" s="3"/>
       <c r="G195" s="3"/>
     </row>
-    <row r="196" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F196" s="3"/>
       <c r="G196" s="3"/>
     </row>
-    <row r="197" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E197" s="3"/>
       <c r="F197" s="3"/>
       <c r="G197" s="3"/>
     </row>
-    <row r="198" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F198" s="3"/>
       <c r="G198" s="3"/>
     </row>
-    <row r="199" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E199" s="3"/>
+    <row r="199" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F199" s="3"/>
       <c r="G199" s="3"/>
     </row>
-    <row r="200" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F200" s="3"/>
       <c r="G200" s="3"/>
     </row>
-    <row r="201" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F201" s="3"/>
       <c r="G201" s="3"/>
     </row>
-    <row r="202" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F202" s="3"/>
       <c r="G202" s="3"/>
     </row>
-    <row r="203" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F203" s="3"/>
       <c r="G203" s="3"/>
     </row>
-    <row r="204" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F204" s="3"/>
       <c r="G204" s="3"/>
     </row>
-    <row r="205" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F205" s="3"/>
       <c r="G205" s="3"/>
     </row>
-    <row r="206" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E206" s="3"/>
       <c r="F206" s="3"/>
       <c r="G206" s="3"/>
     </row>
-    <row r="207" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F207" s="3"/>
       <c r="G207" s="3"/>
     </row>
-    <row r="208" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E208" s="3"/>
+    <row r="208" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F208" s="3"/>
       <c r="G208" s="3"/>
     </row>
-    <row r="209" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F209" s="3"/>
       <c r="G209" s="3"/>
     </row>
-    <row r="210" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F210" s="3"/>
       <c r="G210" s="3"/>
     </row>
-    <row r="211" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F211" s="3"/>
       <c r="G211" s="3"/>
     </row>
-    <row r="212" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F212" s="3"/>
       <c r="G212" s="3"/>
     </row>
-    <row r="213" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F213" s="3"/>
       <c r="G213" s="3"/>
     </row>
-    <row r="214" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F214" s="3"/>
       <c r="G214" s="3"/>
     </row>
-    <row r="215" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E215" s="3"/>
       <c r="F215" s="3"/>
       <c r="G215" s="3"/>
     </row>
-    <row r="216" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F216" s="3"/>
       <c r="G216" s="3"/>
     </row>
-    <row r="217" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E217" s="3"/>
+    <row r="217" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F217" s="3"/>
       <c r="G217" s="3"/>
     </row>
-    <row r="218" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F218" s="3"/>
       <c r="G218" s="3"/>
     </row>
-    <row r="219" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F219" s="3"/>
       <c r="G219" s="3"/>
     </row>
-    <row r="220" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F220" s="3"/>
       <c r="G220" s="3"/>
     </row>
-    <row r="221" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F221" s="3"/>
       <c r="G221" s="3"/>
     </row>
-    <row r="222" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F222" s="3"/>
       <c r="G222" s="3"/>
     </row>
-    <row r="223" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F223" s="3"/>
       <c r="G223" s="3"/>
     </row>
-    <row r="224" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E224" s="3"/>
       <c r="F224" s="3"/>
       <c r="G224" s="3"/>
     </row>
-    <row r="225" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F225" s="3"/>
       <c r="G225" s="3"/>
     </row>
-    <row r="226" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E226" s="3"/>
+    <row r="226" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F226" s="3"/>
       <c r="G226" s="3"/>
     </row>
-    <row r="227" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F227" s="3"/>
       <c r="G227" s="3"/>
     </row>
-    <row r="228" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F228" s="3"/>
       <c r="G228" s="3"/>
     </row>
-    <row r="229" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F229" s="3"/>
       <c r="G229" s="3"/>
     </row>
-    <row r="230" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F230" s="3"/>
       <c r="G230" s="3"/>
     </row>
-    <row r="231" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F231" s="3"/>
       <c r="G231" s="3"/>
     </row>
-    <row r="232" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F232" s="3"/>
       <c r="G232" s="3"/>
     </row>
-    <row r="233" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E233" s="3"/>
       <c r="F233" s="3"/>
       <c r="G233" s="3"/>
     </row>
-    <row r="234" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F234" s="3"/>
       <c r="G234" s="3"/>
     </row>
-    <row r="235" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E235" s="3"/>
+    <row r="235" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F235" s="3"/>
       <c r="G235" s="3"/>
     </row>
-    <row r="236" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F236" s="3"/>
       <c r="G236" s="3"/>
     </row>
-    <row r="237" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F237" s="3"/>
       <c r="G237" s="3"/>
     </row>
-    <row r="238" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F238" s="3"/>
       <c r="G238" s="3"/>
     </row>
-    <row r="239" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F239" s="3"/>
       <c r="G239" s="3"/>
     </row>
-    <row r="240" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F240" s="3"/>
       <c r="G240" s="3"/>
     </row>
-    <row r="241" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F241" s="3"/>
       <c r="G241" s="3"/>
     </row>
-    <row r="242" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E242" s="3"/>
       <c r="F242" s="3"/>
       <c r="G242" s="3"/>
     </row>
-    <row r="243" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F243" s="3"/>
       <c r="G243" s="3"/>
     </row>
-    <row r="244" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E244" s="3"/>
+    <row r="244" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F244" s="3"/>
       <c r="G244" s="3"/>
     </row>
-    <row r="245" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F245" s="3"/>
       <c r="G245" s="3"/>
     </row>
-    <row r="246" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F246" s="3"/>
       <c r="G246" s="3"/>
     </row>
-    <row r="247" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F247" s="3"/>
       <c r="G247" s="3"/>
     </row>
-    <row r="248" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F248" s="3"/>
       <c r="G248" s="3"/>
     </row>
-    <row r="249" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F249" s="3"/>
       <c r="G249" s="3"/>
     </row>
-    <row r="250" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F250" s="3"/>
       <c r="G250" s="3"/>
     </row>
-    <row r="251" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E251" s="3"/>
       <c r="F251" s="3"/>
       <c r="G251" s="3"/>
     </row>
-    <row r="252" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F252" s="3"/>
       <c r="G252" s="3"/>
     </row>
-    <row r="253" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E253" s="3"/>
+    <row r="253" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F253" s="3"/>
       <c r="G253" s="3"/>
     </row>
-    <row r="254" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F254" s="3"/>
       <c r="G254" s="3"/>
     </row>
-    <row r="255" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F255" s="3"/>
       <c r="G255" s="3"/>
     </row>
-    <row r="256" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F256" s="3"/>
       <c r="G256" s="3"/>
     </row>
-    <row r="257" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F257" s="3"/>
       <c r="G257" s="3"/>
     </row>
-    <row r="258" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F258" s="3"/>
       <c r="G258" s="3"/>
     </row>
-    <row r="259" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F259" s="3"/>
       <c r="G259" s="3"/>
     </row>
-    <row r="260" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E260" s="3"/>
       <c r="F260" s="3"/>
       <c r="G260" s="3"/>
     </row>
-    <row r="261" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F261" s="3"/>
       <c r="G261" s="3"/>
     </row>
-    <row r="262" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E262" s="3"/>
+    <row r="262" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F262" s="3"/>
       <c r="G262" s="3"/>
     </row>
-    <row r="263" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F263" s="3"/>
       <c r="G263" s="3"/>
     </row>
-    <row r="264" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F264" s="3"/>
       <c r="G264" s="3"/>
     </row>
-    <row r="265" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F265" s="3"/>
       <c r="G265" s="3"/>
     </row>
-    <row r="266" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F266" s="3"/>
       <c r="G266" s="3"/>
     </row>
-    <row r="267" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F267" s="3"/>
       <c r="G267" s="3"/>
     </row>
-    <row r="268" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F268" s="3"/>
       <c r="G268" s="3"/>
     </row>
-    <row r="269" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E269" s="3"/>
       <c r="F269" s="3"/>
       <c r="G269" s="3"/>
     </row>
-    <row r="270" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F270" s="3"/>
       <c r="G270" s="3"/>
     </row>
-    <row r="271" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E271" s="3"/>
+    <row r="271" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F271" s="3"/>
       <c r="G271" s="3"/>
     </row>
-    <row r="272" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F272" s="3"/>
       <c r="G272" s="3"/>
     </row>
-    <row r="273" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F273" s="3"/>
       <c r="G273" s="3"/>
     </row>
-    <row r="274" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F274" s="3"/>
       <c r="G274" s="3"/>
     </row>
-    <row r="275" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F275" s="3"/>
       <c r="G275" s="3"/>
     </row>
-    <row r="276" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F276" s="3"/>
       <c r="G276" s="3"/>
     </row>
-    <row r="277" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F277" s="3"/>
       <c r="G277" s="3"/>
     </row>
-    <row r="278" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E278" s="3"/>
       <c r="F278" s="3"/>
       <c r="G278" s="3"/>
     </row>
-    <row r="279" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F279" s="3"/>
       <c r="G279" s="3"/>
     </row>
-    <row r="280" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E280" s="3"/>
+    <row r="280" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F280" s="3"/>
       <c r="G280" s="3"/>
     </row>
-    <row r="281" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F281" s="3"/>
       <c r="G281" s="3"/>
     </row>
-    <row r="282" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F282" s="3"/>
-      <c r="G282" s="3"/>
-    </row>
-    <row r="283" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F283" s="3"/>
-      <c r="G283" s="3"/>
-    </row>
-    <row r="284" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F284" s="3"/>
-      <c r="G284" s="3"/>
-    </row>
-    <row r="285" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F285" s="3"/>
-      <c r="G285" s="3"/>
-    </row>
-    <row r="286" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F286" s="3"/>
-      <c r="G286" s="3"/>
-    </row>
-    <row r="287" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F287" s="3"/>
-      <c r="G287" s="3"/>
-    </row>
-    <row r="288" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F288" s="3"/>
-      <c r="G288" s="3"/>
-    </row>
-    <row r="289" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E289" s="3"/>
-      <c r="F289" s="3"/>
-      <c r="G289" s="3"/>
-    </row>
-    <row r="290" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F290" s="3"/>
-      <c r="G290" s="3"/>
-    </row>
-    <row r="291" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F291" s="3"/>
-      <c r="G291" s="3"/>
-    </row>
-    <row r="292" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="F292" s="3"/>
-      <c r="G292" s="3"/>
-    </row>
-    <row r="293" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="294" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="295" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="296" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="297" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="298" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="299" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="300" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="301" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="302" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="303" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="304" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="282" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="283" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="284" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="285" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="286" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="287" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="288" spans="5:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>